<commit_message>
docs(competitor-analysis): fix company count and tighten status flags
- Correct scope wording: 47 competitors across 19 category labels (the
  48th source row is the title banner, not a company) in README + scorecard
- Confluent: state IBM's ~$11B acquisition as COMPLETED (17 Mar 2026,
  verified via IBM newsroom/PR Newswire) instead of "acquiring"; drop the
  weakly-sourced 800-layoffs figure to "reported/unconfirmed"
- Inpher: clarify Arcium took the core tech & team (Nov 2024), not a full
  corporate acquisition
- Ocean Protocol/ASI exit: note the accompanying litigation

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XmpJH9Zvw1ufPHpzKrwV22
</commit_message>
<xml_diff>
--- a/competitor-analysis/competitor_scorecard.xlsx
+++ b/competitor-analysis/competitor_scorecard.xlsx
@@ -3050,7 +3050,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>ACQUIRED by Arcium (Nov 2024); winding down</t>
+          <t>Core tech &amp; team acquired by Arcium (Nov 2024); winding down</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Public (CFLT); NB: IBM acquiring (~$11B, Mar 2026); 800 layoffs Mar 2026</t>
+          <t>Public (CFLT); IBM acquisition COMPLETED ~$11B, 17 Mar 2026 (announced Dec 2025)</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -3588,7 +3588,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Method: 48 competitors across 12 categories were analysed on website positioning (CTAs, keywords,</t>
+          <t>Method: 47 competitors across 19 category labels were analysed on website positioning (CTAs, keywords,</t>
         </is>
       </c>
     </row>

</xml_diff>